<commit_message>
Run CNN model with new cleaned data (22) & plot std data instead of original data
</commit_message>
<xml_diff>
--- a/docs/Models_Evaluation_Summary.xlsx
+++ b/docs/Models_Evaluation_Summary.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Thao Dan\Study\Research\Models\lstm-forecasting-practice1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Thao Dan\Study\Research\Models\lstm-forecasting-practice1\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E5F3160-74F9-4048-B583-9245784CE3E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C5CFB73-FC2D-4329-A2A2-993BD6703463}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9600" yWindow="0" windowWidth="9600" windowHeight="10200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Evaluation Summary" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>Saved Model No.</t>
   </si>
@@ -82,6 +82,18 @@
   </si>
   <si>
     <t>+ Data contain 0</t>
+  </si>
+  <si>
+    <t>CNN</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>Cleaned New Data (2021 + new 2022)</t>
+  </si>
+  <si>
+    <t>Data before 7 A.M. &amp; after 5 P.M. have been removed along with 0s</t>
   </si>
 </sst>
 </file>
@@ -154,7 +166,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -171,10 +183,16 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -468,14 +486,16 @@
     <col min="1" max="1" width="27.1796875" customWidth="1"/>
     <col min="2" max="2" width="17.1328125" customWidth="1"/>
     <col min="3" max="15" width="15.6796875" hidden="1" customWidth="1"/>
-    <col min="16" max="25" width="15.6796875" customWidth="1"/>
+    <col min="16" max="23" width="15.6796875" customWidth="1"/>
+    <col min="24" max="24" width="20.81640625" customWidth="1"/>
+    <col min="25" max="25" width="15.6796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25" s="2" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.95">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
+      <c r="B1" s="8"/>
       <c r="C1" s="4">
         <v>1</v>
       </c>
@@ -547,10 +567,10 @@
       </c>
     </row>
     <row r="2" spans="1:25" s="1" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3"/>
+      <c r="B2" s="8"/>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
@@ -574,14 +594,16 @@
       <c r="U2" s="5"/>
       <c r="V2" s="5"/>
       <c r="W2" s="5"/>
-      <c r="X2" s="5"/>
+      <c r="X2" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="Y2" s="5"/>
     </row>
-    <row r="3" spans="1:25" s="1" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:25" s="1" customFormat="1" ht="33.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
+      <c r="A3" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="3"/>
+      <c r="B3" s="8"/>
       <c r="C3" s="5"/>
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
@@ -605,14 +627,16 @@
       <c r="U3" s="5"/>
       <c r="V3" s="5"/>
       <c r="W3" s="5"/>
-      <c r="X3" s="5"/>
+      <c r="X3" s="7" t="s">
+        <v>21</v>
+      </c>
       <c r="Y3" s="5"/>
     </row>
     <row r="4" spans="1:25" s="1" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="3"/>
+      <c r="B4" s="8"/>
       <c r="C4" s="5"/>
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
@@ -627,7 +651,7 @@
       <c r="N4" s="5"/>
       <c r="O4" s="5"/>
       <c r="P4" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="Q4" s="5"/>
       <c r="R4" s="5"/>
@@ -636,14 +660,16 @@
       <c r="U4" s="5"/>
       <c r="V4" s="5"/>
       <c r="W4" s="5"/>
-      <c r="X4" s="5"/>
+      <c r="X4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="Y4" s="5"/>
     </row>
     <row r="5" spans="1:25" s="1" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="3"/>
+      <c r="B5" s="8"/>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
@@ -667,14 +693,16 @@
       <c r="U5" s="5"/>
       <c r="V5" s="5"/>
       <c r="W5" s="5"/>
-      <c r="X5" s="5"/>
+      <c r="X5" s="5">
+        <v>1</v>
+      </c>
       <c r="Y5" s="5"/>
     </row>
     <row r="6" spans="1:25" s="1" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="5"/>
@@ -698,12 +726,14 @@
       <c r="U6" s="5"/>
       <c r="V6" s="5"/>
       <c r="W6" s="5"/>
-      <c r="X6" s="5"/>
+      <c r="X6" s="5">
+        <v>9.1800000000000007E-2</v>
+      </c>
       <c r="Y6" s="5"/>
     </row>
     <row r="7" spans="1:25" s="1" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A7" s="3"/>
-      <c r="B7" s="6" t="s">
+      <c r="A7" s="8"/>
+      <c r="B7" s="3" t="s">
         <v>7</v>
       </c>
       <c r="C7" s="5"/>
@@ -727,12 +757,14 @@
       <c r="U7" s="5"/>
       <c r="V7" s="5"/>
       <c r="W7" s="5"/>
-      <c r="X7" s="5"/>
+      <c r="X7" s="5">
+        <v>0.68620000000000003</v>
+      </c>
       <c r="Y7" s="5"/>
     </row>
     <row r="8" spans="1:25" s="1" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A8" s="3"/>
-      <c r="B8" s="6" t="s">
+      <c r="A8" s="8"/>
+      <c r="B8" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C8" s="5"/>
@@ -756,12 +788,14 @@
       <c r="U8" s="5"/>
       <c r="V8" s="5"/>
       <c r="W8" s="5"/>
-      <c r="X8" s="5"/>
+      <c r="X8" s="5">
+        <v>2.0461</v>
+      </c>
       <c r="Y8" s="5"/>
     </row>
     <row r="9" spans="1:25" s="1" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A9" s="3"/>
-      <c r="B9" s="6" t="s">
+      <c r="A9" s="8"/>
+      <c r="B9" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C9" s="5"/>
@@ -785,12 +819,14 @@
       <c r="U9" s="5"/>
       <c r="V9" s="5"/>
       <c r="W9" s="5"/>
-      <c r="X9" s="5"/>
+      <c r="X9" s="5">
+        <v>23.9772</v>
+      </c>
       <c r="Y9" s="5"/>
     </row>
     <row r="10" spans="1:25" s="1" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A10" s="3"/>
-      <c r="B10" s="6" t="s">
+      <c r="A10" s="8"/>
+      <c r="B10" s="3" t="s">
         <v>10</v>
       </c>
       <c r="C10" s="5"/>
@@ -814,12 +850,14 @@
       <c r="U10" s="5"/>
       <c r="V10" s="5"/>
       <c r="W10" s="5"/>
-      <c r="X10" s="5"/>
+      <c r="X10" s="5">
+        <v>7.0199999999999999E-2</v>
+      </c>
       <c r="Y10" s="5"/>
     </row>
     <row r="11" spans="1:25" s="1" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A11" s="3"/>
-      <c r="B11" s="6" t="s">
+      <c r="A11" s="8"/>
+      <c r="B11" s="3" t="s">
         <v>11</v>
       </c>
       <c r="C11" s="5"/>
@@ -843,12 +881,14 @@
       <c r="U11" s="5"/>
       <c r="V11" s="5"/>
       <c r="W11" s="5"/>
-      <c r="X11" s="5"/>
+      <c r="X11" s="5">
+        <v>0.52700000000000002</v>
+      </c>
       <c r="Y11" s="5"/>
     </row>
     <row r="12" spans="1:25" s="1" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A12" s="3"/>
-      <c r="B12" s="6" t="s">
+      <c r="A12" s="8"/>
+      <c r="B12" s="3" t="s">
         <v>12</v>
       </c>
       <c r="C12" s="5"/>
@@ -872,12 +912,14 @@
       <c r="U12" s="5"/>
       <c r="V12" s="5"/>
       <c r="W12" s="5"/>
-      <c r="X12" s="5"/>
+      <c r="X12" s="9">
+        <v>0.30407400000000001</v>
+      </c>
       <c r="Y12" s="5"/>
     </row>
     <row r="13" spans="1:25" s="1" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A13" s="3"/>
-      <c r="B13" s="6" t="s">
+      <c r="A13" s="8"/>
+      <c r="B13" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C13" s="5"/>
@@ -901,14 +943,16 @@
       <c r="U13" s="5"/>
       <c r="V13" s="5"/>
       <c r="W13" s="5"/>
-      <c r="X13" s="5"/>
+      <c r="X13" s="9">
+        <v>2.87602</v>
+      </c>
       <c r="Y13" s="5"/>
     </row>
-    <row r="14" spans="1:25" s="1" customFormat="1" ht="42.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="A14" s="3" t="s">
+    <row r="14" spans="1:25" s="1" customFormat="1" ht="61" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
+      <c r="A14" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="3"/>
+      <c r="B14" s="8"/>
       <c r="C14" s="5"/>
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
@@ -922,7 +966,7 @@
       <c r="M14" s="5"/>
       <c r="N14" s="5"/>
       <c r="O14" s="5"/>
-      <c r="P14" s="7" t="s">
+      <c r="P14" s="6" t="s">
         <v>18</v>
       </c>
       <c r="Q14" s="5"/>
@@ -932,7 +976,9 @@
       <c r="U14" s="5"/>
       <c r="V14" s="5"/>
       <c r="W14" s="5"/>
-      <c r="X14" s="5"/>
+      <c r="X14" s="7" t="s">
+        <v>22</v>
+      </c>
       <c r="Y14" s="5"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Run CNN-LSTM models (23)
</commit_message>
<xml_diff>
--- a/docs/Models_Evaluation_Summary.xlsx
+++ b/docs/Models_Evaluation_Summary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Thao Dan\Study\Research\Models\lstm-forecasting-practice1\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C5CFB73-FC2D-4329-A2A2-993BD6703463}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A6F6F6B-8998-43F0-B75B-FA881D4ED39C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9600" yWindow="0" windowWidth="9600" windowHeight="10200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="24">
   <si>
     <t>Saved Model No.</t>
   </si>
@@ -94,12 +94,18 @@
   </si>
   <si>
     <t>Data before 7 A.M. &amp; after 5 P.M. have been removed along with 0s</t>
+  </si>
+  <si>
+    <t>CNN - LSTM</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="169" formatCode="0.0000%"/>
+  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -192,7 +198,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -597,7 +603,9 @@
       <c r="X2" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="Y2" s="5"/>
+      <c r="Y2" s="5" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="3" spans="1:25" s="1" customFormat="1" ht="33.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
       <c r="A3" s="8" t="s">
@@ -630,7 +638,9 @@
       <c r="X3" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="Y3" s="5"/>
+      <c r="Y3" s="7" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="4" spans="1:25" s="1" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
       <c r="A4" s="8" t="s">
@@ -663,7 +673,9 @@
       <c r="X4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="Y4" s="5"/>
+      <c r="Y4" s="5" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="5" spans="1:25" s="1" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
       <c r="A5" s="8" t="s">
@@ -696,7 +708,9 @@
       <c r="X5" s="5">
         <v>1</v>
       </c>
-      <c r="Y5" s="5"/>
+      <c r="Y5" s="5">
+        <v>1</v>
+      </c>
     </row>
     <row r="6" spans="1:25" s="1" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
       <c r="A6" s="8" t="s">
@@ -729,7 +743,9 @@
       <c r="X6" s="5">
         <v>9.1800000000000007E-2</v>
       </c>
-      <c r="Y6" s="5"/>
+      <c r="Y6" s="5">
+        <v>8.3099999999999993E-2</v>
+      </c>
     </row>
     <row r="7" spans="1:25" s="1" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
       <c r="A7" s="8"/>
@@ -760,7 +776,9 @@
       <c r="X7" s="5">
         <v>0.68620000000000003</v>
       </c>
-      <c r="Y7" s="5"/>
+      <c r="Y7" s="5">
+        <v>0.61960000000000004</v>
+      </c>
     </row>
     <row r="8" spans="1:25" s="1" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
       <c r="A8" s="8"/>
@@ -791,7 +809,9 @@
       <c r="X8" s="5">
         <v>2.0461</v>
       </c>
-      <c r="Y8" s="5"/>
+      <c r="Y8" s="5">
+        <v>1.9369000000000001</v>
+      </c>
     </row>
     <row r="9" spans="1:25" s="1" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
       <c r="A9" s="8"/>
@@ -822,7 +842,9 @@
       <c r="X9" s="5">
         <v>23.9772</v>
       </c>
-      <c r="Y9" s="5"/>
+      <c r="Y9" s="5">
+        <v>17.8429</v>
+      </c>
     </row>
     <row r="10" spans="1:25" s="1" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
       <c r="A10" s="8"/>
@@ -853,7 +875,9 @@
       <c r="X10" s="5">
         <v>7.0199999999999999E-2</v>
       </c>
-      <c r="Y10" s="5"/>
+      <c r="Y10" s="5">
+        <v>5.7000000000000002E-2</v>
+      </c>
     </row>
     <row r="11" spans="1:25" s="1" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
       <c r="A11" s="8"/>
@@ -884,7 +908,9 @@
       <c r="X11" s="5">
         <v>0.52700000000000002</v>
       </c>
-      <c r="Y11" s="5"/>
+      <c r="Y11" s="5">
+        <v>0.46610000000000001</v>
+      </c>
     </row>
     <row r="12" spans="1:25" s="1" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
       <c r="A12" s="8"/>
@@ -915,7 +941,9 @@
       <c r="X12" s="9">
         <v>0.30407400000000001</v>
       </c>
-      <c r="Y12" s="5"/>
+      <c r="Y12" s="9">
+        <v>0.26660099999999998</v>
+      </c>
     </row>
     <row r="13" spans="1:25" s="1" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
       <c r="A13" s="8"/>
@@ -946,7 +974,9 @@
       <c r="X13" s="9">
         <v>2.87602</v>
       </c>
-      <c r="Y13" s="5"/>
+      <c r="Y13" s="9">
+        <v>2.615361</v>
+      </c>
     </row>
     <row r="14" spans="1:25" s="1" customFormat="1" ht="61" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
       <c r="A14" s="8" t="s">

</xml_diff>